<commit_message>
all report add export to excel
</commit_message>
<xml_diff>
--- a/public/employee bulk upload.xlsx
+++ b/public/employee bulk upload.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ganesh-harale\standard-device-management\public\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\admin\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -16,15 +16,26 @@
   </sheets>
   <calcPr calcId="152511"/>
   <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+  <si>
+    <t>Sr.No</t>
+  </si>
   <si>
     <t>BioId</t>
   </si>
@@ -32,38 +43,68 @@
     <t>EmpId</t>
   </si>
   <si>
+    <t>FullName</t>
+  </si>
+  <si>
     <t>Category</t>
   </si>
   <si>
     <t>Department</t>
   </si>
   <si>
-    <t>Teaching Staff</t>
-  </si>
-  <si>
-    <t>Software Department</t>
-  </si>
-  <si>
-    <t>Prashant Shinde</t>
-  </si>
-  <si>
-    <t>Branch Name</t>
-  </si>
-  <si>
-    <t>Pune</t>
-  </si>
-  <si>
-    <t>Full Name</t>
+    <t>Branch</t>
+  </si>
+  <si>
+    <t>EmpType(Staff/Contractor)</t>
+  </si>
+  <si>
+    <t>ContractorName</t>
+  </si>
+  <si>
+    <t>Designation</t>
+  </si>
+  <si>
+    <t>Company</t>
+  </si>
+  <si>
+    <t>cardNum</t>
+  </si>
+  <si>
+    <t>accessGroup</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="1" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0;[Red]0"/>
+  </numFmts>
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -89,8 +130,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -151,7 +198,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
+        <a:latin typeface="Calibri Light"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック Light"/>
@@ -186,7 +233,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック"/>
@@ -361,66 +408,71 @@
   </a:themeElements>
   <a:objectDefaults/>
   <a:extraClrSchemeLst/>
-  <a:extLst>
-    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
-    </a:ext>
-  </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:M1"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="3" max="3" width="22" customWidth="1"/>
+    <col min="2" max="2" width="16" style="4" customWidth="1"/>
+    <col min="3" max="3" width="22" style="4" customWidth="1"/>
     <col min="4" max="4" width="18.7109375" customWidth="1"/>
     <col min="5" max="5" width="19.7109375" customWidth="1"/>
     <col min="6" max="6" width="22.7109375" customWidth="1"/>
+    <col min="7" max="7" width="30.5703125" customWidth="1"/>
+    <col min="8" max="8" width="17.85546875" customWidth="1"/>
+    <col min="9" max="9" width="20.42578125" customWidth="1"/>
+    <col min="10" max="10" width="22.42578125" customWidth="1"/>
+    <col min="11" max="11" width="20.28515625" customWidth="1"/>
+    <col min="12" max="12" width="21.42578125" customWidth="1"/>
+    <col min="13" max="13" width="16.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1" spans="1:13">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="D1" t="s">
-        <v>2</v>
-      </c>
-      <c r="E1" t="s">
-        <v>3</v>
-      </c>
-      <c r="F1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2">
-        <v>101</v>
-      </c>
-      <c r="B2">
-        <v>105</v>
-      </c>
-      <c r="C2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D2" t="s">
-        <v>4</v>
-      </c>
-      <c r="E2" t="s">
-        <v>5</v>
-      </c>
-      <c r="F2" t="s">
-        <v>8</v>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="5" t="s">
+        <v>12</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
new requerement changes ganesh
</commit_message>
<xml_diff>
--- a/public/employee bulk upload.xlsx
+++ b/public/employee bulk upload.xlsx
@@ -67,10 +67,10 @@
     <t>Company</t>
   </si>
   <si>
-    <t>cardNum</t>
-  </si>
-  <si>
-    <t>accessGroup</t>
+    <t>Access Group</t>
+  </si>
+  <si>
+    <t>CardNum</t>
   </si>
 </sst>
 </file>
@@ -80,7 +80,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0;[Red]0"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -89,6 +89,7 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -96,13 +97,7 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
+      <b/>
       <sz val="11"/>
       <color rgb="FFFF0000"/>
       <name val="Calibri"/>
@@ -130,14 +125,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -416,8 +409,8 @@
   <dimension ref="A1:M1"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="16" style="4" customWidth="1"/>
-    <col min="3" max="3" width="22" style="4" customWidth="1"/>
+    <col min="2" max="2" width="16" style="1" customWidth="1"/>
+    <col min="3" max="3" width="22" style="1" customWidth="1"/>
     <col min="4" max="4" width="18.7109375" customWidth="1"/>
     <col min="5" max="5" width="19.7109375" customWidth="1"/>
     <col min="6" max="6" width="22.7109375" customWidth="1"/>
@@ -430,8 +423,8 @@
     <col min="13" max="13" width="16.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:13" s="2" customFormat="1">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
@@ -440,35 +433,35 @@
       <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="6" t="s">
+      <c r="I1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="J1" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="K1" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="6" t="s">
+      <c r="L1" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="M1" s="4" t="s">
         <v>11</v>
-      </c>
-      <c r="M1" s="5" t="s">
-        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>